<commit_message>
feat: enhance inventory matching and sample data
Improve sheet detection logic for computer and software inventory, add support for indexed sheet naming, and update sample data formats to prioritize serial/service tag linkage.
</commit_message>
<xml_diff>
--- a/data/sample_data.xlsx
+++ b/data/sample_data.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="Danh Sách Máy Tính" sheetId="1" r:id="rId1"/>
-    <sheet name="Danh Sách Phần Mềm" sheetId="2" r:id="rId2"/>
-    <sheet name="Danh Mục Tiêu Chuẩn (Catalog)" sheetId="3" r:id="rId3"/>
+    <sheet name="1. Danh sach may tinh" sheetId="1" r:id="rId1"/>
+    <sheet name="2. Phan mem" sheetId="2" r:id="rId2"/>
+    <sheet name="3. Danh muc tieu chuan" sheetId="3" r:id="rId3"/>
   </sheets>
 </workbook>
 </file>
@@ -399,262 +399,457 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:L5"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
+        <v>STT</v>
+      </c>
+      <c r="B1" t="str">
         <v>Tên Máy Tính (Hostname)</v>
       </c>
-      <c r="B1" t="str">
+      <c r="C1" t="str">
         <v>Người Sử Dụng</v>
       </c>
-      <c r="C1" t="str">
+      <c r="D1" t="str">
         <v>Phòng Ban</v>
-      </c>
-      <c r="D1" t="str">
-        <v>Số Serial</v>
       </c>
       <c r="E1" t="str">
         <v>Hệ Điều Hành</v>
       </c>
       <c r="F1" t="str">
-        <v>Cấu Hình / Model</v>
+        <v>Model / Cấu Hình Phần Cứng</v>
+      </c>
+      <c r="G1" t="str">
+        <v>Số Serial / Service Tag</v>
+      </c>
+      <c r="H1" t="str">
+        <v>Hãng Sản Xuất</v>
+      </c>
+      <c r="I1" t="str">
+        <v>Vi Xử Lý (CPU)</v>
+      </c>
+      <c r="J1" t="str">
+        <v>Bộ Nhớ RAM</v>
+      </c>
+      <c r="K1" t="str">
+        <v>Ổ Cứng Lưu Trữ</v>
+      </c>
+      <c r="L1" t="str">
+        <v>VGA (Card màn hình)</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="str">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="str">
         <v>KT-DESKTOP-01</v>
       </c>
-      <c r="B2" t="str">
+      <c r="C2" t="str">
         <v>Nguyễn Thị Hoa</v>
       </c>
-      <c r="C2" t="str">
+      <c r="D2" t="str">
         <v>Kế Toán</v>
-      </c>
-      <c r="D2" t="str">
-        <v>DL7090-KT01</v>
       </c>
       <c r="E2" t="str">
         <v>Windows 11 Pro 64-bit</v>
       </c>
       <c r="F2" t="str">
-        <v>Dell OptiPlex 7090 - Core i5, 16GB</v>
+        <v>Dell OptiPlex 7090</v>
+      </c>
+      <c r="G2" t="str">
+        <v>DL7090-KT01</v>
+      </c>
+      <c r="H2" t="str">
+        <v>Dell Inc.</v>
+      </c>
+      <c r="I2" t="str">
+        <v>Intel Core i5-11500 @ 2.70GHz</v>
+      </c>
+      <c r="J2" t="str">
+        <v>16GB DDR4</v>
+      </c>
+      <c r="K2" t="str">
+        <v>512GB NVMe SSD</v>
+      </c>
+      <c r="L2" t="str">
+        <v>Intel UHD Graphics 750</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="str">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" t="str">
         <v>KD-LAPTOP-02</v>
       </c>
-      <c r="B3" t="str">
+      <c r="C3" t="str">
         <v>Trần Văn Nam</v>
       </c>
-      <c r="C3" t="str">
+      <c r="D3" t="str">
         <v>Kinh Doanh</v>
-      </c>
-      <c r="D3" t="str">
-        <v>LNV-T14-KD02</v>
       </c>
       <c r="E3" t="str">
         <v>Windows 10 Pro 64-bit</v>
       </c>
       <c r="F3" t="str">
-        <v>Lenovo ThinkPad T14 - Core i7, 16GB</v>
+        <v>Lenovo ThinkPad T14 Gen 2</v>
+      </c>
+      <c r="G3" t="str">
+        <v>LNV-T14-KD02</v>
+      </c>
+      <c r="H3" t="str">
+        <v>Lenovo</v>
+      </c>
+      <c r="I3" t="str">
+        <v>Intel Core i7-1165G7 @ 2.80GHz</v>
+      </c>
+      <c r="J3" t="str">
+        <v>16GB DDR4</v>
+      </c>
+      <c r="K3" t="str">
+        <v>512GB NVMe SSD</v>
+      </c>
+      <c r="L3" t="str">
+        <v>Intel Iris Xe Graphics</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="str">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" t="str">
         <v>ENG-WORKSTATION-01</v>
       </c>
-      <c r="B4" t="str">
+      <c r="C4" t="str">
         <v>Lê Minh Tuấn</v>
       </c>
-      <c r="C4" t="str">
+      <c r="D4" t="str">
         <v>Kỹ Thuật</v>
       </c>
-      <c r="D4" t="str">
+      <c r="E4" t="str">
+        <v>Windows 11 Pro 64-bit</v>
+      </c>
+      <c r="F4" t="str">
+        <v>Dell Precision 3660</v>
+      </c>
+      <c r="G4" t="str">
         <v>DL3660-ENG01</v>
       </c>
-      <c r="E4" t="str">
-        <v>Windows 11 Pro</v>
-      </c>
-      <c r="F4" t="str">
-        <v>Dell Precision 3660 - Core i9, RTX</v>
+      <c r="H4" t="str">
+        <v>Dell Inc.</v>
+      </c>
+      <c r="I4" t="str">
+        <v>Intel Core i9-12900K @ 3.20GHz</v>
+      </c>
+      <c r="J4" t="str">
+        <v>32GB DDR5</v>
+      </c>
+      <c r="K4" t="str">
+        <v>1TB NVMe SSD + 2TB HDD</v>
+      </c>
+      <c r="L4" t="str">
+        <v>NVIDIA GeForce RTX 4080 16GB</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="str">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" t="str">
         <v>HR-PC-01</v>
       </c>
-      <c r="B5" t="str">
+      <c r="C5" t="str">
         <v>Phạm Thu Trang</v>
       </c>
-      <c r="C5" t="str">
+      <c r="D5" t="str">
         <v>Hành Chính Nhân Sự</v>
-      </c>
-      <c r="D5" t="str">
-        <v>HP400G7-HR01</v>
       </c>
       <c r="E5" t="str">
         <v>Windows 11 Home</v>
       </c>
       <c r="F5" t="str">
-        <v>HP ProDesk 400 G7 - Core i3, 8GB</v>
+        <v>HP ProDesk 400 G7</v>
+      </c>
+      <c r="G5" t="str">
+        <v>HP400G7-HR01</v>
+      </c>
+      <c r="H5" t="str">
+        <v>HP Inc.</v>
+      </c>
+      <c r="I5" t="str">
+        <v>Intel Core i3-10100 @ 3.60GHz</v>
+      </c>
+      <c r="J5" t="str">
+        <v>8GB DDR4</v>
+      </c>
+      <c r="K5" t="str">
+        <v>256GB NVMe SSD</v>
+      </c>
+      <c r="L5" t="str">
+        <v>Intel UHD Graphics 630</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L5"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:K7"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>Tên Máy Tính (Hostname)</v>
+        <v>Serial</v>
       </c>
       <c r="B1" t="str">
-        <v>Tên Phần Mềm</v>
+        <v>Model</v>
       </c>
       <c r="C1" t="str">
-        <v>Hãng SX</v>
+        <v>Tên phần mềm (Name)</v>
       </c>
       <c r="D1" t="str">
-        <v>Phiên Bản</v>
+        <v>Phiên bản (Version)</v>
       </c>
       <c r="E1" t="str">
-        <v>Tình Trạng Hóa Đơn (Có/Chưa)</v>
+        <v>Nhà phát hành (Publisher)</v>
       </c>
       <c r="F1" t="str">
-        <v>Số Hóa Đơn / Ghi Chú</v>
+        <v>Ngày cài (Install Date)</v>
+      </c>
+      <c r="G1" t="str">
+        <v>Dung lượng (Size)</v>
+      </c>
+      <c r="H1" t="str">
+        <v>Kiến trúc</v>
+      </c>
+      <c r="I1" t="str">
+        <v>Phạm vi</v>
+      </c>
+      <c r="J1" t="str">
+        <v>Vị trí cài đặt (Location)</v>
+      </c>
+      <c r="K1" t="str">
+        <v>Chuỗi gỡ cài đặt (Uninstall String)</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>KT-DESKTOP-01</v>
+        <v>DL7090-KT01</v>
       </c>
       <c r="B2" t="str">
+        <v>Dell OptiPlex 7090</v>
+      </c>
+      <c r="C2" t="str">
         <v>Microsoft Office Home &amp; Business 2021</v>
       </c>
-      <c r="C2" t="str">
+      <c r="D2" t="str">
+        <v>16.0.14332.20204</v>
+      </c>
+      <c r="E2" t="str">
         <v>Microsoft Corporation</v>
       </c>
-      <c r="D2" t="str">
-        <v>16.0</v>
-      </c>
-      <c r="E2" t="str">
-        <v>Có</v>
-      </c>
       <c r="F2" t="str">
-        <v>HĐ GTGT #0023412</v>
+        <v>2023-08-15</v>
+      </c>
+      <c r="G2" t="str">
+        <v>3.85 GB</v>
+      </c>
+      <c r="H2" t="str">
+        <v>64-bit</v>
+      </c>
+      <c r="I2" t="str">
+        <v>Machine</v>
+      </c>
+      <c r="J2" t="str">
+        <v>C:\Program Files\Microsoft Office\root\Office16</v>
+      </c>
+      <c r="K2" t="str">
+        <v>MsiExec.exe /X{90160000-0011-0000-1000-0000000FF1CE}</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>KT-DESKTOP-01</v>
+        <v>DL7090-KT01</v>
       </c>
       <c r="B3" t="str">
-        <v>7-Zip</v>
+        <v>Dell OptiPlex 7090</v>
       </c>
       <c r="C3" t="str">
-        <v>Igor Pavlov</v>
+        <v>7-Zip 23.01 (x64)</v>
       </c>
       <c r="D3" t="str">
         <v>23.01</v>
       </c>
       <c r="E3" t="str">
-        <v>FOSS</v>
+        <v>Igor Pavlov</v>
       </c>
       <c r="F3" t="str">
-        <v>FOSS (Không cần HĐ)</v>
+        <v>2023-08-15</v>
+      </c>
+      <c r="G3" t="str">
+        <v>5.2 MB</v>
+      </c>
+      <c r="H3" t="str">
+        <v>64-bit</v>
+      </c>
+      <c r="I3" t="str">
+        <v>Machine</v>
+      </c>
+      <c r="J3" t="str">
+        <v>C:\Program Files\7-Zip</v>
+      </c>
+      <c r="K3" t="str">
+        <v>"C:\Program Files\7-Zip\Uninstall.exe"</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>KT-DESKTOP-01</v>
+        <v>DL7090-KT01</v>
       </c>
       <c r="B4" t="str">
-        <v>WinRAR</v>
+        <v>Dell OptiPlex 7090</v>
       </c>
       <c r="C4" t="str">
+        <v>WinRAR 6.24 (64-bit)</v>
+      </c>
+      <c r="D4" t="str">
+        <v>6.24.0</v>
+      </c>
+      <c r="E4" t="str">
         <v>win.rar GmbH</v>
       </c>
-      <c r="D4" t="str">
-        <v>6.24</v>
-      </c>
-      <c r="E4" t="str">
-        <v>Chưa</v>
-      </c>
       <c r="F4" t="str">
-        <v>Cần gỡ bỏ thay bằng 7-Zip</v>
+        <v>2023-09-02</v>
+      </c>
+      <c r="G4" t="str">
+        <v>9.4 MB</v>
+      </c>
+      <c r="H4" t="str">
+        <v>64-bit</v>
+      </c>
+      <c r="I4" t="str">
+        <v>Machine</v>
+      </c>
+      <c r="J4" t="str">
+        <v>C:\Program Files\WinRAR</v>
+      </c>
+      <c r="K4" t="str">
+        <v>"C:\Program Files\WinRAR\uninstall.exe"</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>KD-LAPTOP-02</v>
+        <v>LNV-T14-KD02</v>
       </c>
       <c r="B5" t="str">
+        <v>Lenovo ThinkPad T14 Gen 2</v>
+      </c>
+      <c r="C5" t="str">
         <v>TeamViewer</v>
       </c>
-      <c r="C5" t="str">
-        <v>TeamViewer Germany</v>
-      </c>
       <c r="D5" t="str">
-        <v>15.48</v>
+        <v>15.48.4</v>
       </c>
       <c r="E5" t="str">
-        <v>Chưa</v>
+        <v>TeamViewer Germany GmbH</v>
       </c>
       <c r="F5" t="str">
-        <v>Bẫy Free cá nhân</v>
+        <v>2023-11-10</v>
+      </c>
+      <c r="G5" t="str">
+        <v>78.2 MB</v>
+      </c>
+      <c r="H5" t="str">
+        <v>64-bit</v>
+      </c>
+      <c r="I5" t="str">
+        <v>Machine</v>
+      </c>
+      <c r="J5" t="str">
+        <v>C:\Program Files\TeamViewer</v>
+      </c>
+      <c r="K5" t="str">
+        <v>"C:\Program Files\TeamViewer\uninstall.exe"</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>ENG-WORKSTATION-01</v>
+        <v>DL3660-ENG01</v>
       </c>
       <c r="B6" t="str">
+        <v>Dell Precision 3660</v>
+      </c>
+      <c r="C6" t="str">
         <v>AutoCAD 2024</v>
       </c>
-      <c r="C6" t="str">
-        <v>Autodesk Inc.</v>
-      </c>
       <c r="D6" t="str">
-        <v>24.3</v>
+        <v>24.3.61.0</v>
       </c>
       <c r="E6" t="str">
-        <v>Chưa</v>
+        <v>Autodesk, Inc.</v>
       </c>
       <c r="F6" t="str">
-        <v>Chưa có bản quyền VAT</v>
+        <v>2023-05-20</v>
+      </c>
+      <c r="G6" t="str">
+        <v>4.12 GB</v>
+      </c>
+      <c r="H6" t="str">
+        <v>64-bit</v>
+      </c>
+      <c r="I6" t="str">
+        <v>Machine</v>
+      </c>
+      <c r="J6" t="str">
+        <v>C:\Program Files\Autodesk\AutoCAD 2024</v>
+      </c>
+      <c r="K6" t="str">
+        <v>"C:\Program Files\Autodesk\AutoCAD 2024\Setup\Setup.exe" /P {ACAD-7101:409} /M ACAD /language en-US</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>ENG-WORKSTATION-01</v>
+        <v>DL3660-ENG01</v>
       </c>
       <c r="B7" t="str">
+        <v>Dell Precision 3660</v>
+      </c>
+      <c r="C7" t="str">
         <v>Phần mềm nội bộ công ty</v>
-      </c>
-      <c r="C7" t="str">
-        <v>Nội bộ</v>
       </c>
       <c r="D7" t="str">
         <v>1.0</v>
       </c>
       <c r="E7" t="str">
-        <v>FOSS</v>
+        <v>Nội bộ công ty</v>
       </c>
       <c r="F7" t="str">
-        <v>Tool viết riêng nội bộ</v>
+        <v>2023-06-01</v>
+      </c>
+      <c r="G7" t="str">
+        <v>45 MB</v>
+      </c>
+      <c r="H7" t="str">
+        <v>64-bit</v>
+      </c>
+      <c r="I7" t="str">
+        <v>Machine</v>
+      </c>
+      <c r="J7" t="str">
+        <v>C:\CompanyApps\InternalTool</v>
+      </c>
+      <c r="K7" t="str">
+        <v>C:\CompanyApps\InternalTool\uninstall.exe</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F7"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K7"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
style: enhance dashboard layout and theme visuals
Add CSS components for cards, ribbons, and pill badges to improve UI structure. Update global background and typography for better readability.
</commit_message>
<xml_diff>
--- a/data/sample_data.xlsx
+++ b/data/sample_data.xlsx
@@ -400,6 +400,20 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:L5"/>
+  <cols>
+    <col min="1" max="1" width="8.83203125" customWidth="1"/>
+    <col min="2" max="2" width="27.83203125" customWidth="1"/>
+    <col min="3" max="3" width="18.83203125" customWidth="1"/>
+    <col min="4" max="4" width="22.83203125" customWidth="1"/>
+    <col min="5" max="5" width="25.83203125" customWidth="1"/>
+    <col min="6" max="6" width="30.83203125" customWidth="1"/>
+    <col min="7" max="7" width="27.83203125" customWidth="1"/>
+    <col min="8" max="8" width="17.83203125" customWidth="1"/>
+    <col min="9" max="9" width="34.83203125" customWidth="1"/>
+    <col min="10" max="10" width="14.83203125" customWidth="1"/>
+    <col min="11" max="11" width="26.83203125" customWidth="1"/>
+    <col min="12" max="12" width="32.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -601,6 +615,19 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:K7"/>
+  <cols>
+    <col min="1" max="1" width="16.83203125" customWidth="1"/>
+    <col min="2" max="2" width="29.83203125" customWidth="1"/>
+    <col min="3" max="3" width="41.83203125" customWidth="1"/>
+    <col min="4" max="4" width="23.83203125" customWidth="1"/>
+    <col min="5" max="5" width="29.83203125" customWidth="1"/>
+    <col min="6" max="6" width="27.83203125" customWidth="1"/>
+    <col min="7" max="7" width="21.83203125" customWidth="1"/>
+    <col min="8" max="8" width="13.83203125" customWidth="1"/>
+    <col min="9" max="9" width="12.83203125" customWidth="1"/>
+    <col min="10" max="10" width="51.83203125" customWidth="1"/>
+    <col min="11" max="11" width="80.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -857,6 +884,20 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:L36"/>
+  <cols>
+    <col min="1" max="1" width="21.83203125" customWidth="1"/>
+    <col min="2" max="2" width="44.83203125" customWidth="1"/>
+    <col min="3" max="3" width="80.83203125" customWidth="1"/>
+    <col min="4" max="4" width="30.83203125" customWidth="1"/>
+    <col min="5" max="5" width="21.83203125" customWidth="1"/>
+    <col min="6" max="6" width="33.83203125" customWidth="1"/>
+    <col min="7" max="7" width="23.83203125" customWidth="1"/>
+    <col min="8" max="8" width="25.83203125" customWidth="1"/>
+    <col min="9" max="9" width="80.83203125" customWidth="1"/>
+    <col min="10" max="10" width="55.83203125" customWidth="1"/>
+    <col min="11" max="11" width="25.83203125" customWidth="1"/>
+    <col min="12" max="12" width="17.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">

</xml_diff>